<commit_message>
Loại hóa đơn mua vào không đứng tên Hưng Mộc
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VfLr1awuTTrH4a4KRG8gM5
</commit_message>
<xml_diff>
--- a/BC_DoanhThu_ChiPhi_Quy3.xlsx
+++ b/BC_DoanhThu_ChiPhi_Quy3.xlsx
@@ -14,7 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cần xác nhận" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Chi phí'!$A$4:$Q$44</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Chi phí'!$A$4:$Q$43</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -66,7 +66,7 @@
       <sz val="13"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -81,11 +81,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F2F2F2"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -115,7 +110,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -137,13 +132,6 @@
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="9" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -616,31 +604,31 @@
         <v/>
       </c>
       <c r="C5" s="5">
-        <f>SUMIFS('Chi phí'!$L$5:$L$44,'Chi phí'!$B$5:$B$44,$A5,'Chi phí'!$O$5:$O$44,C$4,'Chi phí'!$P$5:$P$44,"Có")</f>
+        <f>SUMIFS('Chi phí'!$L$5:$L$43,'Chi phí'!$B$5:$B$43,$A5,'Chi phí'!$O$5:$O$43,C$4,'Chi phí'!$P$5:$P$43,"Có")</f>
         <v/>
       </c>
       <c r="D5" s="5">
-        <f>SUMIFS('Chi phí'!$L$5:$L$44,'Chi phí'!$B$5:$B$44,$A5,'Chi phí'!$O$5:$O$44,D$4,'Chi phí'!$P$5:$P$44,"Có")</f>
+        <f>SUMIFS('Chi phí'!$L$5:$L$43,'Chi phí'!$B$5:$B$43,$A5,'Chi phí'!$O$5:$O$43,D$4,'Chi phí'!$P$5:$P$43,"Có")</f>
         <v/>
       </c>
       <c r="E5" s="5">
-        <f>SUMIFS('Chi phí'!$L$5:$L$44,'Chi phí'!$B$5:$B$44,$A5,'Chi phí'!$O$5:$O$44,E$4,'Chi phí'!$P$5:$P$44,"Có")</f>
+        <f>SUMIFS('Chi phí'!$L$5:$L$43,'Chi phí'!$B$5:$B$43,$A5,'Chi phí'!$O$5:$O$43,E$4,'Chi phí'!$P$5:$P$43,"Có")</f>
         <v/>
       </c>
       <c r="F5" s="5">
-        <f>SUMIFS('Chi phí'!$L$5:$L$44,'Chi phí'!$B$5:$B$44,$A5,'Chi phí'!$O$5:$O$44,F$4,'Chi phí'!$P$5:$P$44,"Có")</f>
+        <f>SUMIFS('Chi phí'!$L$5:$L$43,'Chi phí'!$B$5:$B$43,$A5,'Chi phí'!$O$5:$O$43,F$4,'Chi phí'!$P$5:$P$43,"Có")</f>
         <v/>
       </c>
       <c r="G5" s="5">
-        <f>SUMIFS('Chi phí'!$L$5:$L$44,'Chi phí'!$B$5:$B$44,$A5,'Chi phí'!$O$5:$O$44,G$4,'Chi phí'!$P$5:$P$44,"Có")</f>
+        <f>SUMIFS('Chi phí'!$L$5:$L$43,'Chi phí'!$B$5:$B$43,$A5,'Chi phí'!$O$5:$O$43,G$4,'Chi phí'!$P$5:$P$43,"Có")</f>
         <v/>
       </c>
       <c r="H5" s="5">
-        <f>SUMIFS('Chi phí'!$L$5:$L$44,'Chi phí'!$B$5:$B$44,$A5,'Chi phí'!$O$5:$O$44,H$4,'Chi phí'!$P$5:$P$44,"Có")</f>
+        <f>SUMIFS('Chi phí'!$L$5:$L$43,'Chi phí'!$B$5:$B$43,$A5,'Chi phí'!$O$5:$O$43,H$4,'Chi phí'!$P$5:$P$43,"Có")</f>
         <v/>
       </c>
       <c r="I5" s="5">
-        <f>SUMIFS('Chi phí'!$L$5:$L$44,'Chi phí'!$B$5:$B$44,$A5,'Chi phí'!$O$5:$O$44,I$4,'Chi phí'!$P$5:$P$44,"Có")</f>
+        <f>SUMIFS('Chi phí'!$L$5:$L$43,'Chi phí'!$B$5:$B$43,$A5,'Chi phí'!$O$5:$O$43,I$4,'Chi phí'!$P$5:$P$43,"Có")</f>
         <v/>
       </c>
       <c r="J5" s="5">
@@ -667,31 +655,31 @@
         <v/>
       </c>
       <c r="C6" s="5">
-        <f>SUMIFS('Chi phí'!$L$5:$L$44,'Chi phí'!$B$5:$B$44,$A6,'Chi phí'!$O$5:$O$44,C$4,'Chi phí'!$P$5:$P$44,"Có")</f>
+        <f>SUMIFS('Chi phí'!$L$5:$L$43,'Chi phí'!$B$5:$B$43,$A6,'Chi phí'!$O$5:$O$43,C$4,'Chi phí'!$P$5:$P$43,"Có")</f>
         <v/>
       </c>
       <c r="D6" s="5">
-        <f>SUMIFS('Chi phí'!$L$5:$L$44,'Chi phí'!$B$5:$B$44,$A6,'Chi phí'!$O$5:$O$44,D$4,'Chi phí'!$P$5:$P$44,"Có")</f>
+        <f>SUMIFS('Chi phí'!$L$5:$L$43,'Chi phí'!$B$5:$B$43,$A6,'Chi phí'!$O$5:$O$43,D$4,'Chi phí'!$P$5:$P$43,"Có")</f>
         <v/>
       </c>
       <c r="E6" s="5">
-        <f>SUMIFS('Chi phí'!$L$5:$L$44,'Chi phí'!$B$5:$B$44,$A6,'Chi phí'!$O$5:$O$44,E$4,'Chi phí'!$P$5:$P$44,"Có")</f>
+        <f>SUMIFS('Chi phí'!$L$5:$L$43,'Chi phí'!$B$5:$B$43,$A6,'Chi phí'!$O$5:$O$43,E$4,'Chi phí'!$P$5:$P$43,"Có")</f>
         <v/>
       </c>
       <c r="F6" s="5">
-        <f>SUMIFS('Chi phí'!$L$5:$L$44,'Chi phí'!$B$5:$B$44,$A6,'Chi phí'!$O$5:$O$44,F$4,'Chi phí'!$P$5:$P$44,"Có")</f>
+        <f>SUMIFS('Chi phí'!$L$5:$L$43,'Chi phí'!$B$5:$B$43,$A6,'Chi phí'!$O$5:$O$43,F$4,'Chi phí'!$P$5:$P$43,"Có")</f>
         <v/>
       </c>
       <c r="G6" s="5">
-        <f>SUMIFS('Chi phí'!$L$5:$L$44,'Chi phí'!$B$5:$B$44,$A6,'Chi phí'!$O$5:$O$44,G$4,'Chi phí'!$P$5:$P$44,"Có")</f>
+        <f>SUMIFS('Chi phí'!$L$5:$L$43,'Chi phí'!$B$5:$B$43,$A6,'Chi phí'!$O$5:$O$43,G$4,'Chi phí'!$P$5:$P$43,"Có")</f>
         <v/>
       </c>
       <c r="H6" s="5">
-        <f>SUMIFS('Chi phí'!$L$5:$L$44,'Chi phí'!$B$5:$B$44,$A6,'Chi phí'!$O$5:$O$44,H$4,'Chi phí'!$P$5:$P$44,"Có")</f>
+        <f>SUMIFS('Chi phí'!$L$5:$L$43,'Chi phí'!$B$5:$B$43,$A6,'Chi phí'!$O$5:$O$43,H$4,'Chi phí'!$P$5:$P$43,"Có")</f>
         <v/>
       </c>
       <c r="I6" s="5">
-        <f>SUMIFS('Chi phí'!$L$5:$L$44,'Chi phí'!$B$5:$B$44,$A6,'Chi phí'!$O$5:$O$44,I$4,'Chi phí'!$P$5:$P$44,"Có")</f>
+        <f>SUMIFS('Chi phí'!$L$5:$L$43,'Chi phí'!$B$5:$B$43,$A6,'Chi phí'!$O$5:$O$43,I$4,'Chi phí'!$P$5:$P$43,"Có")</f>
         <v/>
       </c>
       <c r="J6" s="5">
@@ -718,31 +706,31 @@
         <v/>
       </c>
       <c r="C7" s="5">
-        <f>SUMIFS('Chi phí'!$L$5:$L$44,'Chi phí'!$B$5:$B$44,$A7,'Chi phí'!$O$5:$O$44,C$4,'Chi phí'!$P$5:$P$44,"Có")</f>
+        <f>SUMIFS('Chi phí'!$L$5:$L$43,'Chi phí'!$B$5:$B$43,$A7,'Chi phí'!$O$5:$O$43,C$4,'Chi phí'!$P$5:$P$43,"Có")</f>
         <v/>
       </c>
       <c r="D7" s="5">
-        <f>SUMIFS('Chi phí'!$L$5:$L$44,'Chi phí'!$B$5:$B$44,$A7,'Chi phí'!$O$5:$O$44,D$4,'Chi phí'!$P$5:$P$44,"Có")</f>
+        <f>SUMIFS('Chi phí'!$L$5:$L$43,'Chi phí'!$B$5:$B$43,$A7,'Chi phí'!$O$5:$O$43,D$4,'Chi phí'!$P$5:$P$43,"Có")</f>
         <v/>
       </c>
       <c r="E7" s="5">
-        <f>SUMIFS('Chi phí'!$L$5:$L$44,'Chi phí'!$B$5:$B$44,$A7,'Chi phí'!$O$5:$O$44,E$4,'Chi phí'!$P$5:$P$44,"Có")</f>
+        <f>SUMIFS('Chi phí'!$L$5:$L$43,'Chi phí'!$B$5:$B$43,$A7,'Chi phí'!$O$5:$O$43,E$4,'Chi phí'!$P$5:$P$43,"Có")</f>
         <v/>
       </c>
       <c r="F7" s="5">
-        <f>SUMIFS('Chi phí'!$L$5:$L$44,'Chi phí'!$B$5:$B$44,$A7,'Chi phí'!$O$5:$O$44,F$4,'Chi phí'!$P$5:$P$44,"Có")</f>
+        <f>SUMIFS('Chi phí'!$L$5:$L$43,'Chi phí'!$B$5:$B$43,$A7,'Chi phí'!$O$5:$O$43,F$4,'Chi phí'!$P$5:$P$43,"Có")</f>
         <v/>
       </c>
       <c r="G7" s="5">
-        <f>SUMIFS('Chi phí'!$L$5:$L$44,'Chi phí'!$B$5:$B$44,$A7,'Chi phí'!$O$5:$O$44,G$4,'Chi phí'!$P$5:$P$44,"Có")</f>
+        <f>SUMIFS('Chi phí'!$L$5:$L$43,'Chi phí'!$B$5:$B$43,$A7,'Chi phí'!$O$5:$O$43,G$4,'Chi phí'!$P$5:$P$43,"Có")</f>
         <v/>
       </c>
       <c r="H7" s="5">
-        <f>SUMIFS('Chi phí'!$L$5:$L$44,'Chi phí'!$B$5:$B$44,$A7,'Chi phí'!$O$5:$O$44,H$4,'Chi phí'!$P$5:$P$44,"Có")</f>
+        <f>SUMIFS('Chi phí'!$L$5:$L$43,'Chi phí'!$B$5:$B$43,$A7,'Chi phí'!$O$5:$O$43,H$4,'Chi phí'!$P$5:$P$43,"Có")</f>
         <v/>
       </c>
       <c r="I7" s="5">
-        <f>SUMIFS('Chi phí'!$L$5:$L$44,'Chi phí'!$B$5:$B$44,$A7,'Chi phí'!$O$5:$O$44,I$4,'Chi phí'!$P$5:$P$44,"Có")</f>
+        <f>SUMIFS('Chi phí'!$L$5:$L$43,'Chi phí'!$B$5:$B$43,$A7,'Chi phí'!$O$5:$O$43,I$4,'Chi phí'!$P$5:$P$43,"Có")</f>
         <v/>
       </c>
       <c r="J7" s="5">
@@ -769,31 +757,31 @@
         <v/>
       </c>
       <c r="C8" s="5">
-        <f>SUMIFS('Chi phí'!$L$5:$L$44,'Chi phí'!$B$5:$B$44,$A8,'Chi phí'!$O$5:$O$44,C$4,'Chi phí'!$P$5:$P$44,"Có")</f>
+        <f>SUMIFS('Chi phí'!$L$5:$L$43,'Chi phí'!$B$5:$B$43,$A8,'Chi phí'!$O$5:$O$43,C$4,'Chi phí'!$P$5:$P$43,"Có")</f>
         <v/>
       </c>
       <c r="D8" s="5">
-        <f>SUMIFS('Chi phí'!$L$5:$L$44,'Chi phí'!$B$5:$B$44,$A8,'Chi phí'!$O$5:$O$44,D$4,'Chi phí'!$P$5:$P$44,"Có")</f>
+        <f>SUMIFS('Chi phí'!$L$5:$L$43,'Chi phí'!$B$5:$B$43,$A8,'Chi phí'!$O$5:$O$43,D$4,'Chi phí'!$P$5:$P$43,"Có")</f>
         <v/>
       </c>
       <c r="E8" s="5">
-        <f>SUMIFS('Chi phí'!$L$5:$L$44,'Chi phí'!$B$5:$B$44,$A8,'Chi phí'!$O$5:$O$44,E$4,'Chi phí'!$P$5:$P$44,"Có")</f>
+        <f>SUMIFS('Chi phí'!$L$5:$L$43,'Chi phí'!$B$5:$B$43,$A8,'Chi phí'!$O$5:$O$43,E$4,'Chi phí'!$P$5:$P$43,"Có")</f>
         <v/>
       </c>
       <c r="F8" s="5">
-        <f>SUMIFS('Chi phí'!$L$5:$L$44,'Chi phí'!$B$5:$B$44,$A8,'Chi phí'!$O$5:$O$44,F$4,'Chi phí'!$P$5:$P$44,"Có")</f>
+        <f>SUMIFS('Chi phí'!$L$5:$L$43,'Chi phí'!$B$5:$B$43,$A8,'Chi phí'!$O$5:$O$43,F$4,'Chi phí'!$P$5:$P$43,"Có")</f>
         <v/>
       </c>
       <c r="G8" s="5">
-        <f>SUMIFS('Chi phí'!$L$5:$L$44,'Chi phí'!$B$5:$B$44,$A8,'Chi phí'!$O$5:$O$44,G$4,'Chi phí'!$P$5:$P$44,"Có")</f>
+        <f>SUMIFS('Chi phí'!$L$5:$L$43,'Chi phí'!$B$5:$B$43,$A8,'Chi phí'!$O$5:$O$43,G$4,'Chi phí'!$P$5:$P$43,"Có")</f>
         <v/>
       </c>
       <c r="H8" s="5">
-        <f>SUMIFS('Chi phí'!$L$5:$L$44,'Chi phí'!$B$5:$B$44,$A8,'Chi phí'!$O$5:$O$44,H$4,'Chi phí'!$P$5:$P$44,"Có")</f>
+        <f>SUMIFS('Chi phí'!$L$5:$L$43,'Chi phí'!$B$5:$B$43,$A8,'Chi phí'!$O$5:$O$43,H$4,'Chi phí'!$P$5:$P$43,"Có")</f>
         <v/>
       </c>
       <c r="I8" s="5">
-        <f>SUMIFS('Chi phí'!$L$5:$L$44,'Chi phí'!$B$5:$B$44,$A8,'Chi phí'!$O$5:$O$44,I$4,'Chi phí'!$P$5:$P$44,"Có")</f>
+        <f>SUMIFS('Chi phí'!$L$5:$L$43,'Chi phí'!$B$5:$B$43,$A8,'Chi phí'!$O$5:$O$43,I$4,'Chi phí'!$P$5:$P$43,"Có")</f>
         <v/>
       </c>
       <c r="J8" s="5">
@@ -1319,7 +1307,7 @@
         <v/>
       </c>
       <c r="C31" s="5">
-        <f>SUMIFS('Chi phí'!$L$5:$L$44,'Chi phí'!$A$5:$A$44,A31,'Chi phí'!$P$5:$P$44,"Có")</f>
+        <f>SUMIFS('Chi phí'!$L$5:$L$43,'Chi phí'!$A$5:$A$43,A31,'Chi phí'!$P$5:$P$43,"Có")</f>
         <v/>
       </c>
       <c r="D31" s="5">
@@ -1336,7 +1324,7 @@
         <v/>
       </c>
       <c r="C32" s="5">
-        <f>SUMIFS('Chi phí'!$L$5:$L$44,'Chi phí'!$A$5:$A$44,A32,'Chi phí'!$P$5:$P$44,"Có")</f>
+        <f>SUMIFS('Chi phí'!$L$5:$L$43,'Chi phí'!$A$5:$A$43,A32,'Chi phí'!$P$5:$P$43,"Có")</f>
         <v/>
       </c>
       <c r="D32" s="5">
@@ -1353,7 +1341,7 @@
         <v/>
       </c>
       <c r="C33" s="5">
-        <f>SUMIFS('Chi phí'!$L$5:$L$44,'Chi phí'!$A$5:$A$44,A33,'Chi phí'!$P$5:$P$44,"Có")</f>
+        <f>SUMIFS('Chi phí'!$L$5:$L$43,'Chi phí'!$A$5:$A$43,A33,'Chi phí'!$P$5:$P$43,"Có")</f>
         <v/>
       </c>
       <c r="D33" s="5">
@@ -2172,7 +2160,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q46"/>
+  <dimension ref="A1:Q45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2204,7 +2192,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Đơn vị: VNĐ. Cột 'Tính CP' = Không thì dòng bị loại khỏi Tổng hợp. Hóa đơn trùng lặp giữa các thư mục đã được gộp thành 1.</t>
+          <t>Đơn vị: VNĐ. Hóa đơn trùng lặp giữa các thư mục đã được gộp thành 1.</t>
         </is>
       </c>
     </row>
@@ -3380,80 +3368,76 @@
       <c r="Q19" s="14" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="17" t="n">
+      <c r="A20" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="B20" s="17" t="inlineStr">
+      <c r="B20" s="11" t="inlineStr">
         <is>
           <t>AEON – Golden Sea (GS)</t>
         </is>
       </c>
-      <c r="C20" s="17" t="inlineStr">
+      <c r="C20" s="11" t="inlineStr">
         <is>
           <t>Tháng 8/AEON MALL/DCA/VÀO</t>
         </is>
       </c>
-      <c r="D20" s="17" t="inlineStr">
+      <c r="D20" s="11" t="inlineStr">
         <is>
           <t>CTCP Tập đoàn An Phú Cường</t>
         </is>
       </c>
-      <c r="E20" s="17" t="inlineStr">
+      <c r="E20" s="11" t="inlineStr">
         <is>
           <t>2802583021</t>
         </is>
       </c>
-      <c r="F20" s="17" t="inlineStr">
-        <is>
-          <t>00001099</t>
-        </is>
-      </c>
-      <c r="G20" s="17" t="inlineStr">
+      <c r="F20" s="11" t="inlineStr">
+        <is>
+          <t>00001102</t>
+        </is>
+      </c>
+      <c r="G20" s="11" t="inlineStr">
         <is>
           <t>26/08/2026</t>
         </is>
       </c>
-      <c r="H20" s="18" t="inlineStr">
-        <is>
-          <t>Tấm bề mặt LK 3118M F 1220x2440mm</t>
-        </is>
-      </c>
-      <c r="I20" s="17" t="inlineStr">
-        <is>
-          <t>tấm</t>
-        </is>
-      </c>
-      <c r="J20" s="19" t="n">
-        <v>9</v>
-      </c>
-      <c r="K20" s="20" t="n">
-        <v>956818.2</v>
-      </c>
-      <c r="L20" s="20" t="n">
-        <v>8611364</v>
-      </c>
-      <c r="M20" s="21" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="N20" s="20">
+      <c r="H20" s="14" t="inlineStr">
+        <is>
+          <t>Chỉ PVC 9223 23x0.8mm</t>
+        </is>
+      </c>
+      <c r="I20" s="11" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="J20" s="15" t="n">
+        <v>100</v>
+      </c>
+      <c r="K20" s="5" t="n">
+        <v>3700</v>
+      </c>
+      <c r="L20" s="5" t="n">
+        <v>370000</v>
+      </c>
+      <c r="M20" s="16" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="N20" s="5">
         <f>ROUND(L20*M20,0)</f>
         <v/>
       </c>
-      <c r="O20" s="17" t="inlineStr">
-        <is>
-          <t>Ván MDF/Melamine &amp; tấm bề mặt</t>
-        </is>
-      </c>
-      <c r="P20" s="17" t="inlineStr">
-        <is>
-          <t>Không</t>
-        </is>
-      </c>
-      <c r="Q20" s="18" t="inlineStr">
-        <is>
-          <t>HĐ đứng tên người mua là Golden Sea (MST 0314291494), VAT 10% – không phải HĐ đầu vào của Hưng Mộc nên chưa tính vào chi phí</t>
-        </is>
-      </c>
+      <c r="O20" s="11" t="inlineStr">
+        <is>
+          <t>Chỉ/nẹp PVC</t>
+        </is>
+      </c>
+      <c r="P20" s="11" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="Q20" s="14" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="11" t="n">
@@ -3471,42 +3455,42 @@
       </c>
       <c r="D21" s="11" t="inlineStr">
         <is>
-          <t>CTCP Tập đoàn An Phú Cường</t>
+          <t>Cty TNHH Thanh Thùy</t>
         </is>
       </c>
       <c r="E21" s="11" t="inlineStr">
         <is>
-          <t>2802583021</t>
+          <t>3700650344</t>
         </is>
       </c>
       <c r="F21" s="11" t="inlineStr">
         <is>
-          <t>00001102</t>
+          <t>00010949</t>
         </is>
       </c>
       <c r="G21" s="11" t="inlineStr">
         <is>
-          <t>26/08/2026</t>
+          <t>31/08/2026</t>
         </is>
       </c>
       <c r="H21" s="14" t="inlineStr">
         <is>
-          <t>Chỉ PVC 9223 23x0.8mm</t>
+          <t>Ván 9mm kháng ẩm LMR DW MEL 104T 2 mặt 1220x2440</t>
         </is>
       </c>
       <c r="I21" s="11" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>tấm</t>
         </is>
       </c>
       <c r="J21" s="15" t="n">
-        <v>100</v>
+        <v>6</v>
       </c>
       <c r="K21" s="5" t="n">
-        <v>3700</v>
+        <v>392000</v>
       </c>
       <c r="L21" s="5" t="n">
-        <v>370000</v>
+        <v>2352000</v>
       </c>
       <c r="M21" s="16" t="n">
         <v>0.08</v>
@@ -3517,7 +3501,7 @@
       </c>
       <c r="O21" s="11" t="inlineStr">
         <is>
-          <t>Chỉ/nẹp PVC</t>
+          <t>Ván MDF/Melamine &amp; tấm bề mặt</t>
         </is>
       </c>
       <c r="P21" s="11" t="inlineStr">
@@ -3563,22 +3547,22 @@
       </c>
       <c r="H22" s="14" t="inlineStr">
         <is>
-          <t>Ván 9mm kháng ẩm LMR DW MEL 104T 2 mặt 1220x2440</t>
+          <t>Chỉ nẹp 104T 21x0.8</t>
         </is>
       </c>
       <c r="I22" s="11" t="inlineStr">
         <is>
-          <t>tấm</t>
+          <t>m</t>
         </is>
       </c>
       <c r="J22" s="15" t="n">
-        <v>6</v>
+        <v>100</v>
       </c>
       <c r="K22" s="5" t="n">
-        <v>392000</v>
+        <v>1400</v>
       </c>
       <c r="L22" s="5" t="n">
-        <v>2352000</v>
+        <v>140000</v>
       </c>
       <c r="M22" s="16" t="n">
         <v>0.08</v>
@@ -3589,7 +3573,7 @@
       </c>
       <c r="O22" s="11" t="inlineStr">
         <is>
-          <t>Ván MDF/Melamine &amp; tấm bề mặt</t>
+          <t>Chỉ/nẹp PVC</t>
         </is>
       </c>
       <c r="P22" s="11" t="inlineStr">
@@ -3635,7 +3619,7 @@
       </c>
       <c r="H23" s="14" t="inlineStr">
         <is>
-          <t>Chỉ nẹp 104T 21x0.8</t>
+          <t>Chỉ nhựa PVC 21x0.8mm</t>
         </is>
       </c>
       <c r="I23" s="11" t="inlineStr">
@@ -3644,13 +3628,13 @@
         </is>
       </c>
       <c r="J23" s="15" t="n">
-        <v>100</v>
+        <v>400</v>
       </c>
       <c r="K23" s="5" t="n">
-        <v>1400</v>
+        <v>1150</v>
       </c>
       <c r="L23" s="5" t="n">
-        <v>140000</v>
+        <v>460000</v>
       </c>
       <c r="M23" s="16" t="n">
         <v>0.08</v>
@@ -3687,42 +3671,42 @@
       </c>
       <c r="D24" s="11" t="inlineStr">
         <is>
-          <t>Cty TNHH Thanh Thùy</t>
+          <t>Cty TNHH VT TM DV Phượng Hoàng</t>
         </is>
       </c>
       <c r="E24" s="11" t="inlineStr">
         <is>
-          <t>3700650344</t>
+          <t>0305689070</t>
         </is>
       </c>
       <c r="F24" s="11" t="inlineStr">
         <is>
-          <t>00010949</t>
+          <t>00004813</t>
         </is>
       </c>
       <c r="G24" s="11" t="inlineStr">
         <is>
-          <t>31/08/2026</t>
+          <t>28/08/2026</t>
         </is>
       </c>
       <c r="H24" s="14" t="inlineStr">
         <is>
-          <t>Chỉ nhựa PVC 21x0.8mm</t>
+          <t>Cước vận chuyển hàng TP.HCM đi Thanh Hóa (xe 89E-00535)</t>
         </is>
       </c>
       <c r="I24" s="11" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>chuyến</t>
         </is>
       </c>
       <c r="J24" s="15" t="n">
-        <v>400</v>
+        <v>1</v>
       </c>
       <c r="K24" s="5" t="n">
-        <v>1150</v>
+        <v>791667</v>
       </c>
       <c r="L24" s="5" t="n">
-        <v>460000</v>
+        <v>791667</v>
       </c>
       <c r="M24" s="16" t="n">
         <v>0.08</v>
@@ -3733,7 +3717,7 @@
       </c>
       <c r="O24" s="11" t="inlineStr">
         <is>
-          <t>Chỉ/nẹp PVC</t>
+          <t>Vận chuyển</t>
         </is>
       </c>
       <c r="P24" s="11" t="inlineStr">
@@ -3741,11 +3725,15 @@
           <t>Có</t>
         </is>
       </c>
-      <c r="Q24" s="14" t="inlineStr"/>
+      <c r="Q24" s="14" t="inlineStr">
+        <is>
+          <t>HĐ có 3 bản sao ở thư mục Tháng 8 (2 bản) và Tháng 9/GS (1 bản) – chỉ tính 1 lần</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="11" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B25" s="11" t="inlineStr">
         <is>
@@ -3754,12 +3742,12 @@
       </c>
       <c r="C25" s="11" t="inlineStr">
         <is>
-          <t>Tháng 8/AEON MALL/DCA/VÀO</t>
+          <t>Tháng 9/AEON/GS/VÀO</t>
         </is>
       </c>
       <c r="D25" s="11" t="inlineStr">
         <is>
-          <t>Cty TNHH VT TM DV Phượng Hoàng</t>
+          <t>Cty TNHH Vận tải TM DV Phượng Hoàng</t>
         </is>
       </c>
       <c r="E25" s="11" t="inlineStr">
@@ -3769,17 +3757,17 @@
       </c>
       <c r="F25" s="11" t="inlineStr">
         <is>
-          <t>00004813</t>
+          <t>00005001</t>
         </is>
       </c>
       <c r="G25" s="11" t="inlineStr">
         <is>
-          <t>28/08/2026</t>
+          <t>05/09/2026</t>
         </is>
       </c>
       <c r="H25" s="14" t="inlineStr">
         <is>
-          <t>Cước vận chuyển hàng TP.HCM đi Thanh Hóa (xe 89E-00535)</t>
+          <t>Cước vận chuyển hàng TP.HCM đi Thanh Hóa (xe 89C-09217)</t>
         </is>
       </c>
       <c r="I25" s="11" t="inlineStr">
@@ -3791,10 +3779,10 @@
         <v>1</v>
       </c>
       <c r="K25" s="5" t="n">
-        <v>791667</v>
+        <v>625000</v>
       </c>
       <c r="L25" s="5" t="n">
-        <v>791667</v>
+        <v>625000</v>
       </c>
       <c r="M25" s="16" t="n">
         <v>0.08</v>
@@ -3813,11 +3801,7 @@
           <t>Có</t>
         </is>
       </c>
-      <c r="Q25" s="14" t="inlineStr">
-        <is>
-          <t>HĐ có 3 bản sao ở thư mục Tháng 8 (2 bản) và Tháng 9/GS (1 bản) – chỉ tính 1 lần</t>
-        </is>
-      </c>
+      <c r="Q25" s="14" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="11" t="n">
@@ -3835,42 +3819,42 @@
       </c>
       <c r="D26" s="11" t="inlineStr">
         <is>
-          <t>Cty TNHH Vận tải TM DV Phượng Hoàng</t>
+          <t>Cty TNHH SX &amp; TM Kim Mộc</t>
         </is>
       </c>
       <c r="E26" s="11" t="inlineStr">
         <is>
-          <t>0305689070</t>
+          <t>2803198054</t>
         </is>
       </c>
       <c r="F26" s="11" t="inlineStr">
         <is>
-          <t>00005001</t>
+          <t>210</t>
         </is>
       </c>
       <c r="G26" s="11" t="inlineStr">
         <is>
-          <t>05/09/2026</t>
+          <t>10/09/2026</t>
         </is>
       </c>
       <c r="H26" s="14" t="inlineStr">
         <is>
-          <t>Cước vận chuyển hàng TP.HCM đi Thanh Hóa (xe 89C-09217)</t>
+          <t>TPG MDF HMR SP Premium E1 17x1220x2440 216-MN</t>
         </is>
       </c>
       <c r="I26" s="11" t="inlineStr">
         <is>
-          <t>chuyến</t>
+          <t>tấm</t>
         </is>
       </c>
       <c r="J26" s="15" t="n">
-        <v>1</v>
+        <v>37</v>
       </c>
       <c r="K26" s="5" t="n">
-        <v>625000</v>
+        <v>420395.81</v>
       </c>
       <c r="L26" s="5" t="n">
-        <v>625000</v>
+        <v>15554645</v>
       </c>
       <c r="M26" s="16" t="n">
         <v>0.08</v>
@@ -3881,7 +3865,7 @@
       </c>
       <c r="O26" s="11" t="inlineStr">
         <is>
-          <t>Vận chuyển</t>
+          <t>Ván MDF/Melamine &amp; tấm bề mặt</t>
         </is>
       </c>
       <c r="P26" s="11" t="inlineStr">
@@ -3927,7 +3911,7 @@
       </c>
       <c r="H27" s="14" t="inlineStr">
         <is>
-          <t>TPG MDF HMR SP Premium E1 17x1220x2440 216-MN</t>
+          <t>TPG Ván MDF chống ẩm E1 9mm 1138-MN</t>
         </is>
       </c>
       <c r="I27" s="11" t="inlineStr">
@@ -3936,13 +3920,13 @@
         </is>
       </c>
       <c r="J27" s="15" t="n">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="K27" s="5" t="n">
-        <v>420395.81</v>
+        <v>312618.76</v>
       </c>
       <c r="L27" s="5" t="n">
-        <v>15554645</v>
+        <v>8753325</v>
       </c>
       <c r="M27" s="16" t="n">
         <v>0.08</v>
@@ -3999,7 +3983,7 @@
       </c>
       <c r="H28" s="14" t="inlineStr">
         <is>
-          <t>TPG Ván MDF chống ẩm E1 9mm 1138-MN</t>
+          <t>MDF HMR Premium E2 17x1220x2440</t>
         </is>
       </c>
       <c r="I28" s="11" t="inlineStr">
@@ -4008,13 +3992,13 @@
         </is>
       </c>
       <c r="J28" s="15" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="K28" s="5" t="n">
-        <v>312618.76</v>
+        <v>283264.42</v>
       </c>
       <c r="L28" s="5" t="n">
-        <v>8753325</v>
+        <v>8497933</v>
       </c>
       <c r="M28" s="16" t="n">
         <v>0.08</v>
@@ -4071,7 +4055,7 @@
       </c>
       <c r="H29" s="14" t="inlineStr">
         <is>
-          <t>MDF HMR Premium E2 17x1220x2440</t>
+          <t>MDF HMR Premium E2 9x1220x2440</t>
         </is>
       </c>
       <c r="I29" s="11" t="inlineStr">
@@ -4080,13 +4064,13 @@
         </is>
       </c>
       <c r="J29" s="15" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="K29" s="5" t="n">
-        <v>283264.42</v>
+        <v>156441.91</v>
       </c>
       <c r="L29" s="5" t="n">
-        <v>8497933</v>
+        <v>6257676</v>
       </c>
       <c r="M29" s="16" t="n">
         <v>0.08</v>
@@ -4143,22 +4127,22 @@
       </c>
       <c r="H30" s="14" t="inlineStr">
         <is>
-          <t>MDF HMR Premium E2 9x1220x2440</t>
+          <t>Nẹp PVC vân gỗ 1x21x90mm</t>
         </is>
       </c>
       <c r="I30" s="11" t="inlineStr">
         <is>
-          <t>tấm</t>
+          <t>cuộn</t>
         </is>
       </c>
       <c r="J30" s="15" t="n">
-        <v>40</v>
+        <v>21</v>
       </c>
       <c r="K30" s="5" t="n">
-        <v>156441.91</v>
+        <v>87652.64</v>
       </c>
       <c r="L30" s="5" t="n">
-        <v>6257676</v>
+        <v>1840705</v>
       </c>
       <c r="M30" s="16" t="n">
         <v>0.08</v>
@@ -4169,7 +4153,7 @@
       </c>
       <c r="O30" s="11" t="inlineStr">
         <is>
-          <t>Ván MDF/Melamine &amp; tấm bề mặt</t>
+          <t>Chỉ/nẹp PVC</t>
         </is>
       </c>
       <c r="P30" s="11" t="inlineStr">
@@ -4215,7 +4199,7 @@
       </c>
       <c r="H31" s="14" t="inlineStr">
         <is>
-          <t>Nẹp PVC vân gỗ 1x21x90mm</t>
+          <t>Nẹp PVC vân gỗ 1x44x90mm</t>
         </is>
       </c>
       <c r="I31" s="11" t="inlineStr">
@@ -4224,13 +4208,13 @@
         </is>
       </c>
       <c r="J31" s="15" t="n">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="K31" s="5" t="n">
-        <v>87652.64</v>
+        <v>174293.79</v>
       </c>
       <c r="L31" s="5" t="n">
-        <v>1840705</v>
+        <v>1742938</v>
       </c>
       <c r="M31" s="16" t="n">
         <v>0.08</v>
@@ -4267,42 +4251,42 @@
       </c>
       <c r="D32" s="11" t="inlineStr">
         <is>
-          <t>Cty TNHH SX &amp; TM Kim Mộc</t>
+          <t>Cty TNHH Hoàng Hưng Pro</t>
         </is>
       </c>
       <c r="E32" s="11" t="inlineStr">
         <is>
-          <t>2803198054</t>
+          <t>2802454435</t>
         </is>
       </c>
       <c r="F32" s="11" t="inlineStr">
         <is>
-          <t>210</t>
+          <t>00004830</t>
         </is>
       </c>
       <c r="G32" s="11" t="inlineStr">
         <is>
-          <t>10/09/2026</t>
+          <t>08/09/2026</t>
         </is>
       </c>
       <c r="H32" s="14" t="inlineStr">
         <is>
-          <t>Nẹp PVC vân gỗ 1x44x90mm</t>
+          <t>Mica TQ 1220x2440x4.8mm</t>
         </is>
       </c>
       <c r="I32" s="11" t="inlineStr">
         <is>
-          <t>cuộn</t>
+          <t>tấm</t>
         </is>
       </c>
       <c r="J32" s="15" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="K32" s="5" t="n">
-        <v>174293.79</v>
+        <v>663889</v>
       </c>
       <c r="L32" s="5" t="n">
-        <v>1742938</v>
+        <v>663889</v>
       </c>
       <c r="M32" s="16" t="n">
         <v>0.08</v>
@@ -4313,7 +4297,7 @@
       </c>
       <c r="O32" s="11" t="inlineStr">
         <is>
-          <t>Chỉ/nẹp PVC</t>
+          <t>Mica, nhựa, keo &amp; vật tư phụ</t>
         </is>
       </c>
       <c r="P32" s="11" t="inlineStr">
@@ -4359,7 +4343,7 @@
       </c>
       <c r="H33" s="14" t="inlineStr">
         <is>
-          <t>Mica TQ 1220x2440x4.8mm</t>
+          <t>Mica FS000 1220x2440x4.8mm</t>
         </is>
       </c>
       <c r="I33" s="11" t="inlineStr">
@@ -4371,10 +4355,10 @@
         <v>1</v>
       </c>
       <c r="K33" s="5" t="n">
-        <v>663889</v>
+        <v>1467593</v>
       </c>
       <c r="L33" s="5" t="n">
-        <v>663889</v>
+        <v>1467593</v>
       </c>
       <c r="M33" s="16" t="n">
         <v>0.08</v>
@@ -4431,7 +4415,7 @@
       </c>
       <c r="H34" s="14" t="inlineStr">
         <is>
-          <t>Mica FS000 1220x2440x4.8mm</t>
+          <t>Tấm PVC CNC 1220x2440x8mm</t>
         </is>
       </c>
       <c r="I34" s="11" t="inlineStr">
@@ -4440,13 +4424,13 @@
         </is>
       </c>
       <c r="J34" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K34" s="5" t="n">
-        <v>1467593</v>
+        <v>361111</v>
       </c>
       <c r="L34" s="5" t="n">
-        <v>1467593</v>
+        <v>722222</v>
       </c>
       <c r="M34" s="16" t="n">
         <v>0.08</v>
@@ -4503,22 +4487,22 @@
       </c>
       <c r="H35" s="14" t="inlineStr">
         <is>
-          <t>Tấm PVC CNC 1220x2440x8mm</t>
+          <t>Keo silicon Apollo Sealant A500</t>
         </is>
       </c>
       <c r="I35" s="11" t="inlineStr">
         <is>
-          <t>tấm</t>
+          <t>chai</t>
         </is>
       </c>
       <c r="J35" s="15" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K35" s="5" t="n">
-        <v>361111</v>
+        <v>46296.25</v>
       </c>
       <c r="L35" s="5" t="n">
-        <v>722222</v>
+        <v>185185</v>
       </c>
       <c r="M35" s="16" t="n">
         <v>0.08</v>
@@ -4565,32 +4549,32 @@
       </c>
       <c r="F36" s="11" t="inlineStr">
         <is>
-          <t>00004830</t>
+          <t>00004871</t>
         </is>
       </c>
       <c r="G36" s="11" t="inlineStr">
         <is>
-          <t>08/09/2026</t>
+          <t>09/09/2026</t>
         </is>
       </c>
       <c r="H36" s="14" t="inlineStr">
         <is>
-          <t>Keo silicon Apollo Sealant A500</t>
+          <t>Mica TQ 1220x2440x4.8mm</t>
         </is>
       </c>
       <c r="I36" s="11" t="inlineStr">
         <is>
-          <t>chai</t>
+          <t>tấm</t>
         </is>
       </c>
       <c r="J36" s="15" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="K36" s="5" t="n">
-        <v>46296.25</v>
+        <v>663889</v>
       </c>
       <c r="L36" s="5" t="n">
-        <v>185185</v>
+        <v>663889</v>
       </c>
       <c r="M36" s="16" t="n">
         <v>0.08</v>
@@ -4637,32 +4621,32 @@
       </c>
       <c r="F37" s="11" t="inlineStr">
         <is>
-          <t>00004871</t>
+          <t>00004920</t>
         </is>
       </c>
       <c r="G37" s="11" t="inlineStr">
         <is>
-          <t>09/09/2026</t>
+          <t>12/09/2026</t>
         </is>
       </c>
       <c r="H37" s="14" t="inlineStr">
         <is>
-          <t>Mica TQ 1220x2440x4.8mm</t>
+          <t>Tấm nhựa Polycarbonate đặc</t>
         </is>
       </c>
       <c r="I37" s="11" t="inlineStr">
         <is>
-          <t>tấm</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="J37" s="15" t="n">
-        <v>1</v>
+        <v>2.62</v>
       </c>
       <c r="K37" s="5" t="n">
-        <v>663889</v>
+        <v>314532.06</v>
       </c>
       <c r="L37" s="5" t="n">
-        <v>663889</v>
+        <v>824074</v>
       </c>
       <c r="M37" s="16" t="n">
         <v>0.08</v>
@@ -4685,59 +4669,59 @@
     </row>
     <row r="38">
       <c r="A38" s="11" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B38" s="11" t="inlineStr">
         <is>
-          <t>AEON – Golden Sea (GS)</t>
+          <t>AEON – Nhóm Thống (Taco + ICO)</t>
         </is>
       </c>
       <c r="C38" s="11" t="inlineStr">
         <is>
-          <t>Tháng 9/AEON/GS/VÀO</t>
+          <t>Tháng 8/AEON MALL/THỐNG</t>
         </is>
       </c>
       <c r="D38" s="11" t="inlineStr">
         <is>
-          <t>Cty TNHH Hoàng Hưng Pro</t>
+          <t>Cty TNHH KD &amp; TM Huy Tiến</t>
         </is>
       </c>
       <c r="E38" s="11" t="inlineStr">
         <is>
-          <t>2802454435</t>
+          <t>2802839259</t>
         </is>
       </c>
       <c r="F38" s="11" t="inlineStr">
         <is>
-          <t>00004920</t>
+          <t>00000368</t>
         </is>
       </c>
       <c r="G38" s="11" t="inlineStr">
         <is>
-          <t>12/09/2026</t>
+          <t>28/08/2026</t>
         </is>
       </c>
       <c r="H38" s="14" t="inlineStr">
         <is>
-          <t>Tấm nhựa Polycarbonate đặc</t>
+          <t>Nhôm thanh STĐ</t>
         </is>
       </c>
       <c r="I38" s="11" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="J38" s="15" t="n">
-        <v>2.62</v>
+        <v>116.38</v>
       </c>
       <c r="K38" s="5" t="n">
-        <v>314532.06</v>
+        <v>115999.31</v>
       </c>
       <c r="L38" s="5" t="n">
-        <v>824074</v>
+        <v>13500000</v>
       </c>
       <c r="M38" s="16" t="n">
-        <v>0.08</v>
+        <v>0.1</v>
       </c>
       <c r="N38" s="5">
         <f>ROUND(L38*M38,0)</f>
@@ -4745,7 +4729,7 @@
       </c>
       <c r="O38" s="11" t="inlineStr">
         <is>
-          <t>Mica, nhựa, keo &amp; vật tư phụ</t>
+          <t>Nhôm – sắt</t>
         </is>
       </c>
       <c r="P38" s="11" t="inlineStr">
@@ -4771,45 +4755,45 @@
       </c>
       <c r="D39" s="11" t="inlineStr">
         <is>
-          <t>Cty TNHH KD &amp; TM Huy Tiến</t>
+          <t>Cty TNHH Cửa kính Thái Bình</t>
         </is>
       </c>
       <c r="E39" s="11" t="inlineStr">
         <is>
-          <t>2802839259</t>
+          <t>2803078776</t>
         </is>
       </c>
       <c r="F39" s="11" t="inlineStr">
         <is>
-          <t>00000368</t>
+          <t>31</t>
         </is>
       </c>
       <c r="G39" s="11" t="inlineStr">
         <is>
-          <t>28/08/2026</t>
+          <t>26/08/2026</t>
         </is>
       </c>
       <c r="H39" s="14" t="inlineStr">
         <is>
-          <t>Nhôm thanh STĐ</t>
+          <t>Kính cường lực 10mm trà đỏ</t>
         </is>
       </c>
       <c r="I39" s="11" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="J39" s="15" t="n">
-        <v>116.38</v>
+        <v>6.03</v>
       </c>
       <c r="K39" s="5" t="n">
-        <v>115999.31</v>
+        <v>734400</v>
       </c>
       <c r="L39" s="5" t="n">
-        <v>13500000</v>
+        <v>4428432</v>
       </c>
       <c r="M39" s="16" t="n">
-        <v>0.1</v>
+        <v>0.08</v>
       </c>
       <c r="N39" s="5">
         <f>ROUND(L39*M39,0)</f>
@@ -4817,7 +4801,7 @@
       </c>
       <c r="O39" s="11" t="inlineStr">
         <is>
-          <t>Nhôm – sắt</t>
+          <t>Kính cường lực</t>
         </is>
       </c>
       <c r="P39" s="11" t="inlineStr">
@@ -4863,7 +4847,7 @@
       </c>
       <c r="H40" s="14" t="inlineStr">
         <is>
-          <t>Kính cường lực 10mm trà đỏ</t>
+          <t>Kính cường lực 10mm trắng</t>
         </is>
       </c>
       <c r="I40" s="11" t="inlineStr">
@@ -4872,13 +4856,13 @@
         </is>
       </c>
       <c r="J40" s="15" t="n">
-        <v>6.03</v>
+        <v>34.5</v>
       </c>
       <c r="K40" s="5" t="n">
-        <v>734400</v>
+        <v>318625.804</v>
       </c>
       <c r="L40" s="5" t="n">
-        <v>4428432</v>
+        <v>10992590</v>
       </c>
       <c r="M40" s="16" t="n">
         <v>0.08</v>
@@ -4901,7 +4885,7 @@
     </row>
     <row r="41">
       <c r="A41" s="11" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B41" s="11" t="inlineStr">
         <is>
@@ -4910,32 +4894,32 @@
       </c>
       <c r="C41" s="11" t="inlineStr">
         <is>
-          <t>Tháng 8/AEON MALL/THỐNG</t>
+          <t>Tháng 9/AEON/THỐNG/VÀO</t>
         </is>
       </c>
       <c r="D41" s="11" t="inlineStr">
         <is>
-          <t>Cty TNHH Cửa kính Thái Bình</t>
+          <t>Cty TNHH Tú Tươi (CN Thanh Hóa)</t>
         </is>
       </c>
       <c r="E41" s="11" t="inlineStr">
         <is>
-          <t>2803078776</t>
+          <t>2803184132</t>
         </is>
       </c>
       <c r="F41" s="11" t="inlineStr">
         <is>
-          <t>31</t>
+          <t>125</t>
         </is>
       </c>
       <c r="G41" s="11" t="inlineStr">
         <is>
-          <t>26/08/2026</t>
+          <t>04/09/2026</t>
         </is>
       </c>
       <c r="H41" s="14" t="inlineStr">
         <is>
-          <t>Kính cường lực 10mm trắng</t>
+          <t>Kính CL 10mm trắng</t>
         </is>
       </c>
       <c r="I41" s="11" t="inlineStr">
@@ -4944,13 +4928,13 @@
         </is>
       </c>
       <c r="J41" s="15" t="n">
-        <v>34.5</v>
+        <v>84.18000000000001</v>
       </c>
       <c r="K41" s="5" t="n">
-        <v>318625.804</v>
+        <v>220000</v>
       </c>
       <c r="L41" s="5" t="n">
-        <v>10992590</v>
+        <v>18519600</v>
       </c>
       <c r="M41" s="16" t="n">
         <v>0.08</v>
@@ -4987,27 +4971,27 @@
       </c>
       <c r="D42" s="11" t="inlineStr">
         <is>
-          <t>Cty TNHH Tú Tươi (CN Thanh Hóa)</t>
+          <t>Cty TNHH TM &amp; SX Đức Thắng</t>
         </is>
       </c>
       <c r="E42" s="11" t="inlineStr">
         <is>
-          <t>2803184132</t>
+          <t>2801874821</t>
         </is>
       </c>
       <c r="F42" s="11" t="inlineStr">
         <is>
-          <t>125</t>
+          <t>730</t>
         </is>
       </c>
       <c r="G42" s="11" t="inlineStr">
         <is>
-          <t>04/09/2026</t>
+          <t>15/09/2026</t>
         </is>
       </c>
       <c r="H42" s="14" t="inlineStr">
         <is>
-          <t>Kính CL 10mm trắng</t>
+          <t>Kính cường lực 10 ly</t>
         </is>
       </c>
       <c r="I42" s="11" t="inlineStr">
@@ -5016,13 +5000,13 @@
         </is>
       </c>
       <c r="J42" s="15" t="n">
-        <v>84.18000000000001</v>
+        <v>55.556</v>
       </c>
       <c r="K42" s="5" t="n">
-        <v>220000</v>
+        <v>250000</v>
       </c>
       <c r="L42" s="5" t="n">
-        <v>18519600</v>
+        <v>13889000</v>
       </c>
       <c r="M42" s="16" t="n">
         <v>0.08</v>
@@ -5049,52 +5033,52 @@
       </c>
       <c r="B43" s="11" t="inlineStr">
         <is>
-          <t>AEON – Nhóm Thống (Taco + ICO)</t>
+          <t>Moly (Hua Long)</t>
         </is>
       </c>
       <c r="C43" s="11" t="inlineStr">
         <is>
-          <t>Tháng 9/AEON/THỐNG/VÀO</t>
+          <t>Tháng 9/MOLY/VÀO</t>
         </is>
       </c>
       <c r="D43" s="11" t="inlineStr">
         <is>
-          <t>Cty TNHH TM &amp; SX Đức Thắng</t>
+          <t>Cty TNHH SX – TM Đông Á</t>
         </is>
       </c>
       <c r="E43" s="11" t="inlineStr">
         <is>
-          <t>2801874821</t>
+          <t>2801613442</t>
         </is>
       </c>
       <c r="F43" s="11" t="inlineStr">
         <is>
-          <t>730</t>
+          <t>00012909</t>
         </is>
       </c>
       <c r="G43" s="11" t="inlineStr">
         <is>
-          <t>15/09/2026</t>
+          <t>16/09/2026</t>
         </is>
       </c>
       <c r="H43" s="14" t="inlineStr">
         <is>
-          <t>Kính cường lực 10 ly</t>
+          <t>Tủ mát Sanaky VH6009HP</t>
         </is>
       </c>
       <c r="I43" s="11" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>cái</t>
         </is>
       </c>
       <c r="J43" s="15" t="n">
-        <v>55.556</v>
+        <v>1</v>
       </c>
       <c r="K43" s="5" t="n">
-        <v>250000</v>
+        <v>15324074</v>
       </c>
       <c r="L43" s="5" t="n">
-        <v>13889000</v>
+        <v>15324074</v>
       </c>
       <c r="M43" s="16" t="n">
         <v>0.08</v>
@@ -5105,7 +5089,7 @@
       </c>
       <c r="O43" s="11" t="inlineStr">
         <is>
-          <t>Kính cường lực</t>
+          <t>Hàng hóa mua bán (thiết bị)</t>
         </is>
       </c>
       <c r="P43" s="11" t="inlineStr">
@@ -5116,76 +5100,33 @@
       <c r="Q43" s="14" t="inlineStr"/>
     </row>
     <row r="44">
-      <c r="A44" s="11" t="n">
-        <v>9</v>
-      </c>
-      <c r="B44" s="11" t="inlineStr">
-        <is>
-          <t>Moly (Hua Long)</t>
-        </is>
-      </c>
-      <c r="C44" s="11" t="inlineStr">
-        <is>
-          <t>Tháng 9/MOLY/VÀO</t>
-        </is>
-      </c>
-      <c r="D44" s="11" t="inlineStr">
-        <is>
-          <t>Cty TNHH SX – TM Đông Á</t>
-        </is>
-      </c>
-      <c r="E44" s="11" t="inlineStr">
-        <is>
-          <t>2801613442</t>
-        </is>
-      </c>
-      <c r="F44" s="11" t="inlineStr">
-        <is>
-          <t>00012909</t>
-        </is>
-      </c>
-      <c r="G44" s="11" t="inlineStr">
-        <is>
-          <t>16/09/2026</t>
-        </is>
-      </c>
-      <c r="H44" s="14" t="inlineStr">
-        <is>
-          <t>Tủ mát Sanaky VH6009HP</t>
-        </is>
-      </c>
-      <c r="I44" s="11" t="inlineStr">
-        <is>
-          <t>cái</t>
-        </is>
-      </c>
-      <c r="J44" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="K44" s="5" t="n">
-        <v>15324074</v>
-      </c>
-      <c r="L44" s="5" t="n">
-        <v>15324074</v>
-      </c>
-      <c r="M44" s="16" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="N44" s="5">
-        <f>ROUND(L44*M44,0)</f>
-        <v/>
-      </c>
-      <c r="O44" s="11" t="inlineStr">
-        <is>
-          <t>Hàng hóa mua bán (thiết bị)</t>
-        </is>
-      </c>
-      <c r="P44" s="11" t="inlineStr">
-        <is>
-          <t>Có</t>
-        </is>
-      </c>
-      <c r="Q44" s="14" t="inlineStr"/>
+      <c r="A44" s="12" t="n"/>
+      <c r="B44" s="12" t="n"/>
+      <c r="C44" s="12" t="n"/>
+      <c r="D44" s="12" t="n"/>
+      <c r="E44" s="12" t="n"/>
+      <c r="F44" s="12" t="n"/>
+      <c r="G44" s="12" t="n"/>
+      <c r="H44" s="12" t="inlineStr">
+        <is>
+          <t>TỔNG CỘNG (tất cả dòng)</t>
+        </is>
+      </c>
+      <c r="I44" s="12" t="n"/>
+      <c r="J44" s="12" t="n"/>
+      <c r="K44" s="12" t="n"/>
+      <c r="L44" s="7">
+        <f>SUM(L5:L43)</f>
+        <v/>
+      </c>
+      <c r="M44" s="12" t="n"/>
+      <c r="N44" s="7">
+        <f>SUM(N5:N43)</f>
+        <v/>
+      </c>
+      <c r="O44" s="12" t="n"/>
+      <c r="P44" s="12" t="n"/>
+      <c r="Q44" s="12" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="12" t="n"/>
@@ -5197,56 +5138,27 @@
       <c r="G45" s="12" t="n"/>
       <c r="H45" s="12" t="inlineStr">
         <is>
-          <t>TỔNG CỘNG (tất cả dòng)</t>
+          <t>Trong đó tính vào chi phí</t>
         </is>
       </c>
       <c r="I45" s="12" t="n"/>
       <c r="J45" s="12" t="n"/>
       <c r="K45" s="12" t="n"/>
       <c r="L45" s="7">
-        <f>SUM(L5:L44)</f>
+        <f>SUMIFS(L5:L43,P5:P43,"Có")</f>
         <v/>
       </c>
       <c r="M45" s="12" t="n"/>
       <c r="N45" s="7">
-        <f>SUM(N5:N44)</f>
+        <f>SUMIFS(N5:N43,P5:P43,"Có")</f>
         <v/>
       </c>
       <c r="O45" s="12" t="n"/>
       <c r="P45" s="12" t="n"/>
       <c r="Q45" s="12" t="n"/>
     </row>
-    <row r="46">
-      <c r="A46" s="12" t="n"/>
-      <c r="B46" s="12" t="n"/>
-      <c r="C46" s="12" t="n"/>
-      <c r="D46" s="12" t="n"/>
-      <c r="E46" s="12" t="n"/>
-      <c r="F46" s="12" t="n"/>
-      <c r="G46" s="12" t="n"/>
-      <c r="H46" s="12" t="inlineStr">
-        <is>
-          <t>Trong đó tính vào chi phí</t>
-        </is>
-      </c>
-      <c r="I46" s="12" t="n"/>
-      <c r="J46" s="12" t="n"/>
-      <c r="K46" s="12" t="n"/>
-      <c r="L46" s="7">
-        <f>SUMIFS(L5:L44,P5:P44,"Có")</f>
-        <v/>
-      </c>
-      <c r="M46" s="12" t="n"/>
-      <c r="N46" s="7">
-        <f>SUMIFS(N5:N44,P5:P44,"Có")</f>
-        <v/>
-      </c>
-      <c r="O46" s="12" t="n"/>
-      <c r="P46" s="12" t="n"/>
-      <c r="Q46" s="12" t="n"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A4:Q44"/>
+  <autoFilter ref="A4:Q43"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5257,7 +5169,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H32"/>
+  <dimension ref="A1:H31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -5345,7 +5257,7 @@
         <v>2160000</v>
       </c>
       <c r="G4" s="5">
-        <f>SUMIFS('Chi phí'!$L$5:$L$44,'Chi phí'!$F$5:$F$44,B4)</f>
+        <f>SUMIFS('Chi phí'!$L$5:$L$43,'Chi phí'!$F$5:$F$43,B4)</f>
         <v/>
       </c>
       <c r="H4" s="5">
@@ -5379,7 +5291,7 @@
         <v>24753600</v>
       </c>
       <c r="G5" s="5">
-        <f>SUMIFS('Chi phí'!$L$5:$L$44,'Chi phí'!$F$5:$F$44,B5)</f>
+        <f>SUMIFS('Chi phí'!$L$5:$L$43,'Chi phí'!$F$5:$F$43,B5)</f>
         <v/>
       </c>
       <c r="H5" s="5">
@@ -5413,7 +5325,7 @@
         <v>9428400</v>
       </c>
       <c r="G6" s="5">
-        <f>SUMIFS('Chi phí'!$L$5:$L$44,'Chi phí'!$F$5:$F$44,B6)</f>
+        <f>SUMIFS('Chi phí'!$L$5:$L$43,'Chi phí'!$F$5:$F$43,B6)</f>
         <v/>
       </c>
       <c r="H6" s="5">
@@ -5447,7 +5359,7 @@
         <v>6339600</v>
       </c>
       <c r="G7" s="5">
-        <f>SUMIFS('Chi phí'!$L$5:$L$44,'Chi phí'!$F$5:$F$44,B7)</f>
+        <f>SUMIFS('Chi phí'!$L$5:$L$43,'Chi phí'!$F$5:$F$43,B7)</f>
         <v/>
       </c>
       <c r="H7" s="5">
@@ -5481,7 +5393,7 @@
         <v>604800</v>
       </c>
       <c r="G8" s="5">
-        <f>SUMIFS('Chi phí'!$L$5:$L$44,'Chi phí'!$F$5:$F$44,B8)</f>
+        <f>SUMIFS('Chi phí'!$L$5:$L$43,'Chi phí'!$F$5:$F$43,B8)</f>
         <v/>
       </c>
       <c r="H8" s="5">
@@ -5515,7 +5427,7 @@
         <v>4401000</v>
       </c>
       <c r="G9" s="5">
-        <f>SUMIFS('Chi phí'!$L$5:$L$44,'Chi phí'!$F$5:$F$44,B9)</f>
+        <f>SUMIFS('Chi phí'!$L$5:$L$43,'Chi phí'!$F$5:$F$43,B9)</f>
         <v/>
       </c>
       <c r="H9" s="5">
@@ -5549,7 +5461,7 @@
         <v>604800</v>
       </c>
       <c r="G10" s="5">
-        <f>SUMIFS('Chi phí'!$L$5:$L$44,'Chi phí'!$F$5:$F$44,B10)</f>
+        <f>SUMIFS('Chi phí'!$L$5:$L$43,'Chi phí'!$F$5:$F$43,B10)</f>
         <v/>
       </c>
       <c r="H10" s="5">
@@ -5583,7 +5495,7 @@
         <v>3110400</v>
       </c>
       <c r="G11" s="5">
-        <f>SUMIFS('Chi phí'!$L$5:$L$44,'Chi phí'!$F$5:$F$44,B11)</f>
+        <f>SUMIFS('Chi phí'!$L$5:$L$43,'Chi phí'!$F$5:$F$43,B11)</f>
         <v/>
       </c>
       <c r="H11" s="5">
@@ -5599,7 +5511,7 @@
       </c>
       <c r="B12" s="11" t="inlineStr">
         <is>
-          <t>00001099</t>
+          <t>00001102</t>
         </is>
       </c>
       <c r="C12" s="11" t="inlineStr">
@@ -5608,16 +5520,16 @@
         </is>
       </c>
       <c r="D12" s="5" t="n">
-        <v>8611364</v>
+        <v>370000</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>861136</v>
+        <v>29600</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>9472500</v>
+        <v>399600</v>
       </c>
       <c r="G12" s="5">
-        <f>SUMIFS('Chi phí'!$L$5:$L$44,'Chi phí'!$F$5:$F$44,B12)</f>
+        <f>SUMIFS('Chi phí'!$L$5:$L$43,'Chi phí'!$F$5:$F$43,B12)</f>
         <v/>
       </c>
       <c r="H12" s="5">
@@ -5633,25 +5545,25 @@
       </c>
       <c r="B13" s="11" t="inlineStr">
         <is>
-          <t>00001102</t>
+          <t>00010949</t>
         </is>
       </c>
       <c r="C13" s="11" t="inlineStr">
         <is>
-          <t>CTCP Tập đoàn An Phú Cường</t>
+          <t>Cty TNHH Thanh Thùy</t>
         </is>
       </c>
       <c r="D13" s="5" t="n">
-        <v>370000</v>
+        <v>2952000</v>
       </c>
       <c r="E13" s="5" t="n">
-        <v>29600</v>
+        <v>236160</v>
       </c>
       <c r="F13" s="5" t="n">
-        <v>399600</v>
+        <v>3188160</v>
       </c>
       <c r="G13" s="5">
-        <f>SUMIFS('Chi phí'!$L$5:$L$44,'Chi phí'!$F$5:$F$44,B13)</f>
+        <f>SUMIFS('Chi phí'!$L$5:$L$43,'Chi phí'!$F$5:$F$43,B13)</f>
         <v/>
       </c>
       <c r="H13" s="5">
@@ -5667,25 +5579,25 @@
       </c>
       <c r="B14" s="11" t="inlineStr">
         <is>
-          <t>00010949</t>
+          <t>00004813</t>
         </is>
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
-          <t>Cty TNHH Thanh Thùy</t>
+          <t>Cty TNHH VT TM DV Phượng Hoàng</t>
         </is>
       </c>
       <c r="D14" s="5" t="n">
-        <v>2952000</v>
+        <v>791667</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>236160</v>
+        <v>63333</v>
       </c>
       <c r="F14" s="5" t="n">
-        <v>3188160</v>
+        <v>855000</v>
       </c>
       <c r="G14" s="5">
-        <f>SUMIFS('Chi phí'!$L$5:$L$44,'Chi phí'!$F$5:$F$44,B14)</f>
+        <f>SUMIFS('Chi phí'!$L$5:$L$43,'Chi phí'!$F$5:$F$43,B14)</f>
         <v/>
       </c>
       <c r="H14" s="5">
@@ -5701,25 +5613,25 @@
       </c>
       <c r="B15" s="11" t="inlineStr">
         <is>
-          <t>00004813</t>
+          <t>00005001</t>
         </is>
       </c>
       <c r="C15" s="11" t="inlineStr">
         <is>
-          <t>Cty TNHH VT TM DV Phượng Hoàng</t>
+          <t>Cty TNHH Vận tải TM DV Phượng Hoàng</t>
         </is>
       </c>
       <c r="D15" s="5" t="n">
-        <v>791667</v>
+        <v>625000</v>
       </c>
       <c r="E15" s="5" t="n">
-        <v>63333</v>
+        <v>50000</v>
       </c>
       <c r="F15" s="5" t="n">
-        <v>855000</v>
+        <v>675000</v>
       </c>
       <c r="G15" s="5">
-        <f>SUMIFS('Chi phí'!$L$5:$L$44,'Chi phí'!$F$5:$F$44,B15)</f>
+        <f>SUMIFS('Chi phí'!$L$5:$L$43,'Chi phí'!$F$5:$F$43,B15)</f>
         <v/>
       </c>
       <c r="H15" s="5">
@@ -5735,25 +5647,25 @@
       </c>
       <c r="B16" s="11" t="inlineStr">
         <is>
-          <t>00005001</t>
+          <t>210</t>
         </is>
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>Cty TNHH Vận tải TM DV Phượng Hoàng</t>
+          <t>Cty TNHH SX &amp; TM Kim Mộc</t>
         </is>
       </c>
       <c r="D16" s="5" t="n">
-        <v>625000</v>
+        <v>42647222</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>50000</v>
+        <v>3411778</v>
       </c>
       <c r="F16" s="5" t="n">
-        <v>675000</v>
+        <v>46059000</v>
       </c>
       <c r="G16" s="5">
-        <f>SUMIFS('Chi phí'!$L$5:$L$44,'Chi phí'!$F$5:$F$44,B16)</f>
+        <f>SUMIFS('Chi phí'!$L$5:$L$43,'Chi phí'!$F$5:$F$43,B16)</f>
         <v/>
       </c>
       <c r="H16" s="5">
@@ -5769,25 +5681,25 @@
       </c>
       <c r="B17" s="11" t="inlineStr">
         <is>
-          <t>210</t>
+          <t>00004830</t>
         </is>
       </c>
       <c r="C17" s="11" t="inlineStr">
         <is>
-          <t>Cty TNHH SX &amp; TM Kim Mộc</t>
+          <t>Cty TNHH Hoàng Hưng Pro</t>
         </is>
       </c>
       <c r="D17" s="5" t="n">
-        <v>42647222</v>
+        <v>3038889</v>
       </c>
       <c r="E17" s="5" t="n">
-        <v>3411778</v>
+        <v>243111</v>
       </c>
       <c r="F17" s="5" t="n">
-        <v>46059000</v>
+        <v>3282000</v>
       </c>
       <c r="G17" s="5">
-        <f>SUMIFS('Chi phí'!$L$5:$L$44,'Chi phí'!$F$5:$F$44,B17)</f>
+        <f>SUMIFS('Chi phí'!$L$5:$L$43,'Chi phí'!$F$5:$F$43,B17)</f>
         <v/>
       </c>
       <c r="H17" s="5">
@@ -5803,7 +5715,7 @@
       </c>
       <c r="B18" s="11" t="inlineStr">
         <is>
-          <t>00004830</t>
+          <t>00004871</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
@@ -5812,16 +5724,16 @@
         </is>
       </c>
       <c r="D18" s="5" t="n">
-        <v>3038889</v>
+        <v>663889</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>243111</v>
+        <v>53111</v>
       </c>
       <c r="F18" s="5" t="n">
-        <v>3282000</v>
+        <v>717000</v>
       </c>
       <c r="G18" s="5">
-        <f>SUMIFS('Chi phí'!$L$5:$L$44,'Chi phí'!$F$5:$F$44,B18)</f>
+        <f>SUMIFS('Chi phí'!$L$5:$L$43,'Chi phí'!$F$5:$F$43,B18)</f>
         <v/>
       </c>
       <c r="H18" s="5">
@@ -5837,7 +5749,7 @@
       </c>
       <c r="B19" s="11" t="inlineStr">
         <is>
-          <t>00004871</t>
+          <t>00004920</t>
         </is>
       </c>
       <c r="C19" s="11" t="inlineStr">
@@ -5846,16 +5758,16 @@
         </is>
       </c>
       <c r="D19" s="5" t="n">
-        <v>663889</v>
+        <v>824074</v>
       </c>
       <c r="E19" s="5" t="n">
-        <v>53111</v>
+        <v>65926</v>
       </c>
       <c r="F19" s="5" t="n">
-        <v>717000</v>
+        <v>890000</v>
       </c>
       <c r="G19" s="5">
-        <f>SUMIFS('Chi phí'!$L$5:$L$44,'Chi phí'!$F$5:$F$44,B19)</f>
+        <f>SUMIFS('Chi phí'!$L$5:$L$43,'Chi phí'!$F$5:$F$43,B19)</f>
         <v/>
       </c>
       <c r="H19" s="5">
@@ -5871,25 +5783,25 @@
       </c>
       <c r="B20" s="11" t="inlineStr">
         <is>
-          <t>00004920</t>
+          <t>00000368</t>
         </is>
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t>Cty TNHH Hoàng Hưng Pro</t>
+          <t>Cty TNHH KD &amp; TM Huy Tiến</t>
         </is>
       </c>
       <c r="D20" s="5" t="n">
-        <v>824074</v>
+        <v>13500000</v>
       </c>
       <c r="E20" s="5" t="n">
-        <v>65926</v>
+        <v>1350000</v>
       </c>
       <c r="F20" s="5" t="n">
-        <v>890000</v>
+        <v>14850000</v>
       </c>
       <c r="G20" s="5">
-        <f>SUMIFS('Chi phí'!$L$5:$L$44,'Chi phí'!$F$5:$F$44,B20)</f>
+        <f>SUMIFS('Chi phí'!$L$5:$L$43,'Chi phí'!$F$5:$F$43,B20)</f>
         <v/>
       </c>
       <c r="H20" s="5">
@@ -5905,25 +5817,25 @@
       </c>
       <c r="B21" s="11" t="inlineStr">
         <is>
-          <t>00000368</t>
+          <t>31</t>
         </is>
       </c>
       <c r="C21" s="11" t="inlineStr">
         <is>
-          <t>Cty TNHH KD &amp; TM Huy Tiến</t>
+          <t>Cty TNHH Cửa kính Thái Bình</t>
         </is>
       </c>
       <c r="D21" s="5" t="n">
-        <v>13500000</v>
+        <v>15421022</v>
       </c>
       <c r="E21" s="5" t="n">
-        <v>1350000</v>
+        <v>1233682</v>
       </c>
       <c r="F21" s="5" t="n">
-        <v>14850000</v>
+        <v>16654704</v>
       </c>
       <c r="G21" s="5">
-        <f>SUMIFS('Chi phí'!$L$5:$L$44,'Chi phí'!$F$5:$F$44,B21)</f>
+        <f>SUMIFS('Chi phí'!$L$5:$L$43,'Chi phí'!$F$5:$F$43,B21)</f>
         <v/>
       </c>
       <c r="H21" s="5">
@@ -5939,25 +5851,25 @@
       </c>
       <c r="B22" s="11" t="inlineStr">
         <is>
-          <t>31</t>
+          <t>125</t>
         </is>
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
-          <t>Cty TNHH Cửa kính Thái Bình</t>
+          <t>Cty TNHH Tú Tươi (CN Thanh Hóa)</t>
         </is>
       </c>
       <c r="D22" s="5" t="n">
-        <v>15421022</v>
+        <v>18519600</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>1233682</v>
+        <v>1481568</v>
       </c>
       <c r="F22" s="5" t="n">
-        <v>16654704</v>
+        <v>20001168</v>
       </c>
       <c r="G22" s="5">
-        <f>SUMIFS('Chi phí'!$L$5:$L$44,'Chi phí'!$F$5:$F$44,B22)</f>
+        <f>SUMIFS('Chi phí'!$L$5:$L$43,'Chi phí'!$F$5:$F$43,B22)</f>
         <v/>
       </c>
       <c r="H22" s="5">
@@ -5973,25 +5885,25 @@
       </c>
       <c r="B23" s="11" t="inlineStr">
         <is>
-          <t>125</t>
+          <t>730</t>
         </is>
       </c>
       <c r="C23" s="11" t="inlineStr">
         <is>
-          <t>Cty TNHH Tú Tươi (CN Thanh Hóa)</t>
+          <t>Cty TNHH TM &amp; SX Đức Thắng</t>
         </is>
       </c>
       <c r="D23" s="5" t="n">
-        <v>18519600</v>
+        <v>13889000</v>
       </c>
       <c r="E23" s="5" t="n">
-        <v>1481568</v>
+        <v>1111120</v>
       </c>
       <c r="F23" s="5" t="n">
-        <v>20001168</v>
+        <v>15000120</v>
       </c>
       <c r="G23" s="5">
-        <f>SUMIFS('Chi phí'!$L$5:$L$44,'Chi phí'!$F$5:$F$44,B23)</f>
+        <f>SUMIFS('Chi phí'!$L$5:$L$43,'Chi phí'!$F$5:$F$43,B23)</f>
         <v/>
       </c>
       <c r="H23" s="5">
@@ -6007,25 +5919,25 @@
       </c>
       <c r="B24" s="11" t="inlineStr">
         <is>
-          <t>730</t>
+          <t>00012909</t>
         </is>
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
-          <t>Cty TNHH TM &amp; SX Đức Thắng</t>
+          <t>Cty TNHH SX – TM Đông Á</t>
         </is>
       </c>
       <c r="D24" s="5" t="n">
-        <v>13889000</v>
+        <v>15324074</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>1111120</v>
+        <v>1225926</v>
       </c>
       <c r="F24" s="5" t="n">
-        <v>15000120</v>
+        <v>16550000</v>
       </c>
       <c r="G24" s="5">
-        <f>SUMIFS('Chi phí'!$L$5:$L$44,'Chi phí'!$F$5:$F$44,B24)</f>
+        <f>SUMIFS('Chi phí'!$L$5:$L$43,'Chi phí'!$F$5:$F$43,B24)</f>
         <v/>
       </c>
       <c r="H24" s="5">
@@ -6036,30 +5948,30 @@
     <row r="25">
       <c r="A25" s="11" t="inlineStr">
         <is>
-          <t>Mua vào</t>
+          <t>Bán ra</t>
         </is>
       </c>
       <c r="B25" s="11" t="inlineStr">
         <is>
-          <t>00012909</t>
+          <t>10</t>
         </is>
       </c>
       <c r="C25" s="11" t="inlineStr">
         <is>
-          <t>Cty TNHH SX – TM Đông Á</t>
+          <t>CTCP Smart Shopping Thanh Hóa</t>
         </is>
       </c>
       <c r="D25" s="5" t="n">
-        <v>15324074</v>
+        <v>6018519</v>
       </c>
       <c r="E25" s="5" t="n">
-        <v>1225926</v>
+        <v>481481</v>
       </c>
       <c r="F25" s="5" t="n">
-        <v>16550000</v>
+        <v>6500000</v>
       </c>
       <c r="G25" s="5">
-        <f>SUMIFS('Chi phí'!$L$5:$L$44,'Chi phí'!$F$5:$F$44,B25)</f>
+        <f>SUMIFS('Doanh thu'!$L$5:$L$14,'Doanh thu'!$E$5:$E$14,B25)</f>
         <v/>
       </c>
       <c r="H25" s="5">
@@ -6075,22 +5987,22 @@
       </c>
       <c r="B26" s="11" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="C26" s="11" t="inlineStr">
         <is>
-          <t>CTCP Smart Shopping Thanh Hóa</t>
+          <t>Cty TNHH XD &amp; DV TM Taco</t>
         </is>
       </c>
       <c r="D26" s="5" t="n">
-        <v>6018519</v>
+        <v>26784900</v>
       </c>
       <c r="E26" s="5" t="n">
-        <v>481481</v>
+        <v>2142792</v>
       </c>
       <c r="F26" s="5" t="n">
-        <v>6500000</v>
+        <v>28927692</v>
       </c>
       <c r="G26" s="5">
         <f>SUMIFS('Doanh thu'!$L$5:$L$14,'Doanh thu'!$E$5:$E$14,B26)</f>
@@ -6109,22 +6021,22 @@
       </c>
       <c r="B27" s="11" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>15</t>
         </is>
       </c>
       <c r="C27" s="11" t="inlineStr">
         <is>
-          <t>Cty TNHH XD &amp; DV TM Taco</t>
+          <t>Cty TNHH XD &amp; TM ICO</t>
         </is>
       </c>
       <c r="D27" s="5" t="n">
-        <v>26784900</v>
+        <v>10466182</v>
       </c>
       <c r="E27" s="5" t="n">
-        <v>2142792</v>
+        <v>1046618</v>
       </c>
       <c r="F27" s="5" t="n">
-        <v>28927692</v>
+        <v>11512800</v>
       </c>
       <c r="G27" s="5">
         <f>SUMIFS('Doanh thu'!$L$5:$L$14,'Doanh thu'!$E$5:$E$14,B27)</f>
@@ -6143,22 +6055,22 @@
       </c>
       <c r="B28" s="11" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>14</t>
         </is>
       </c>
       <c r="C28" s="11" t="inlineStr">
         <is>
-          <t>Cty TNHH XD &amp; TM ICO</t>
+          <t>Cty TNHH ĐT TM DV Golden Sea</t>
         </is>
       </c>
       <c r="D28" s="5" t="n">
-        <v>10466182</v>
+        <v>295887500</v>
       </c>
       <c r="E28" s="5" t="n">
-        <v>1046618</v>
+        <v>23671000</v>
       </c>
       <c r="F28" s="5" t="n">
-        <v>11512800</v>
+        <v>319558500</v>
       </c>
       <c r="G28" s="5">
         <f>SUMIFS('Doanh thu'!$L$5:$L$14,'Doanh thu'!$E$5:$E$14,B28)</f>
@@ -6177,22 +6089,22 @@
       </c>
       <c r="B29" s="11" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>16</t>
         </is>
       </c>
       <c r="C29" s="11" t="inlineStr">
         <is>
-          <t>Cty TNHH ĐT TM DV Golden Sea</t>
+          <t>Cty TNHH Hua Long Moly Việt Nam</t>
         </is>
       </c>
       <c r="D29" s="5" t="n">
-        <v>295887500</v>
+        <v>17731481</v>
       </c>
       <c r="E29" s="5" t="n">
-        <v>23671000</v>
+        <v>1418519</v>
       </c>
       <c r="F29" s="5" t="n">
-        <v>319558500</v>
+        <v>19150000</v>
       </c>
       <c r="G29" s="5">
         <f>SUMIFS('Doanh thu'!$L$5:$L$14,'Doanh thu'!$E$5:$E$14,B29)</f>
@@ -6203,42 +6115,8 @@
         <v/>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="11" t="inlineStr">
-        <is>
-          <t>Bán ra</t>
-        </is>
-      </c>
-      <c r="B30" s="11" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
-      </c>
-      <c r="C30" s="11" t="inlineStr">
-        <is>
-          <t>Cty TNHH Hua Long Moly Việt Nam</t>
-        </is>
-      </c>
-      <c r="D30" s="5" t="n">
-        <v>17731481</v>
-      </c>
-      <c r="E30" s="5" t="n">
-        <v>1418519</v>
-      </c>
-      <c r="F30" s="5" t="n">
-        <v>19150000</v>
-      </c>
-      <c r="G30" s="5">
-        <f>SUMIFS('Doanh thu'!$L$5:$L$14,'Doanh thu'!$E$5:$E$14,B30)</f>
-        <v/>
-      </c>
-      <c r="H30" s="5">
-        <f>G30-D30</f>
-        <v/>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="2" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
         <is>
           <t>Chênh lệch ≤ 2 đồng là do làm tròn trên hóa đơn gốc.</t>
         </is>
@@ -6297,19 +6175,19 @@
       <c r="A4" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="22" t="inlineStr">
-        <is>
-          <t>Hóa đơn An Phú Cường số 00001099 đứng tên Golden Sea</t>
+      <c r="B4" s="17" t="inlineStr">
+        <is>
+          <t>Đã loại hóa đơn không phải của Hưng Mộc</t>
         </is>
       </c>
       <c r="C4" s="14" t="inlineStr">
         <is>
-          <t>Người mua trên HĐ là Golden Sea (MST 0314291494), VAT 10%, trị giá trước thuế 8.611.364. Nằm trong thư mục mua vào của Hưng Mộc.</t>
+          <t>HĐ An Phú Cường số 00001099 (26/08/2026, 8.611.364 trước thuế) có người mua là Golden Sea (MST 0314291494), không phải Hưng Mộc. Đã kiểm tra 24 HĐ mua vào còn lại, tất cả đứng tên Hưng Mộc (MST 2803104433).</t>
         </is>
       </c>
       <c r="D4" s="14" t="inlineStr">
         <is>
-          <t>Em để dòng này ở sheet Chi phí (tô vàng) nhưng đặt 'Tính CP' = Không, nên chưa cộng vào chi phí. Nếu thực tế Hưng Mộc đã trả tiền thì chị đổi thành 'Có'.</t>
+          <t>Đã loại hẳn khỏi sheet Chi phí và Tổng hợp.</t>
         </is>
       </c>
     </row>
@@ -6317,7 +6195,7 @@
       <c r="A5" s="14" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="22" t="inlineStr">
+      <c r="B5" s="17" t="inlineStr">
         <is>
           <t>Doanh thu GS lệch bảng quyết toán đợt 1</t>
         </is>
@@ -6337,7 +6215,7 @@
       <c r="A6" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="22" t="inlineStr">
+      <c r="B6" s="17" t="inlineStr">
         <is>
           <t>Chi phí của GS đang vượt xa doanh thu đã xuất</t>
         </is>
@@ -6357,7 +6235,7 @@
       <c r="A7" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="22" t="inlineStr">
+      <c r="B7" s="17" t="inlineStr">
         <is>
           <t>Chi phí nhóm Thống không có hóa đơn thép hộp</t>
         </is>
@@ -6377,7 +6255,7 @@
       <c r="A8" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="B8" s="22" t="inlineStr">
+      <c r="B8" s="17" t="inlineStr">
         <is>
           <t>Thư mục 'DCA' tháng 7, 8</t>
         </is>
@@ -6397,7 +6275,7 @@
       <c r="A9" s="14" t="n">
         <v>6</v>
       </c>
-      <c r="B9" s="22" t="inlineStr">
+      <c r="B9" s="17" t="inlineStr">
         <is>
           <t>Hóa đơn trùng lặp giữa các thư mục</t>
         </is>
@@ -6417,7 +6295,7 @@
       <c r="A10" s="14" t="n">
         <v>7</v>
       </c>
-      <c r="B10" s="22" t="inlineStr">
+      <c r="B10" s="17" t="inlineStr">
         <is>
           <t>SSTH (Smart Shopping) chưa có chi phí</t>
         </is>
@@ -6437,7 +6315,7 @@
       <c r="A11" s="14" t="n">
         <v>8</v>
       </c>
-      <c r="B11" s="22" t="inlineStr">
+      <c r="B11" s="17" t="inlineStr">
         <is>
           <t>HĐ bán số 13 (ICO) đã thay thế</t>
         </is>
@@ -6457,7 +6335,7 @@
       <c r="A12" s="14" t="n">
         <v>9</v>
       </c>
-      <c r="B12" s="22" t="inlineStr">
+      <c r="B12" s="17" t="inlineStr">
         <is>
           <t>Tên hàng trên HĐ vận chuyển/kính</t>
         </is>

</xml_diff>